<commit_message>
fix(templates): actualizar plantillas de recepcion de muestras y limpieza de archivos temporales
</commit_message>
<xml_diff>
--- a/app/templates/Recepciones/F-LEM-P-01.04 V05 RECEPCIÓN DE MUESTRAS DE ROCA.xlsx
+++ b/app/templates/Recepciones/F-LEM-P-01.04 V05 RECEPCIÓN DE MUESTRAS DE ROCA.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E5AD45-D916-4853-867F-9E274A47D7A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F465790-13C5-47A2-A86E-4B7836BD021E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="975" yWindow="1635" windowWidth="14820" windowHeight="13575" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SEG. ENSAYOS" sheetId="5" r:id="rId1"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="45">
   <si>
     <t>:</t>
   </si>
@@ -228,9 +228,6 @@
     <t>Firma del laboratorio:</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
     <t>DIRECCION DEL SOLICITANTE O CORREO DEL SOLICITANTE</t>
   </si>
   <si>
@@ -246,7 +243,7 @@
     <numFmt numFmtId="165" formatCode="000&quot;-23&quot;"/>
     <numFmt numFmtId="166" formatCode="000&quot;-RO-23&quot;"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -402,8 +399,20 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="10.7"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -574,7 +583,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -726,25 +735,6 @@
     <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -784,49 +774,45 @@
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="2" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -881,79 +867,118 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="16" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1092,9 +1117,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1132,9 +1157,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1167,26 +1192,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1219,26 +1227,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1413,35 +1404,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="19.140625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="1.7109375" style="5" customWidth="1"/>
-    <col min="4" max="4" width="3.42578125" style="5" customWidth="1"/>
-    <col min="5" max="6" width="14.7109375" style="5" customWidth="1"/>
-    <col min="7" max="7" width="11.7109375" style="13" customWidth="1"/>
-    <col min="8" max="8" width="15.28515625" style="5" customWidth="1"/>
-    <col min="9" max="10" width="10.5703125" style="5" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" style="5" customWidth="1"/>
-    <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="6.109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="1.6640625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="3.44140625" style="5" customWidth="1"/>
+    <col min="5" max="6" width="14.6640625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" style="13" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" style="5" customWidth="1"/>
+    <col min="9" max="10" width="10.5546875" style="5" customWidth="1"/>
+    <col min="11" max="11" width="11.6640625" style="5" customWidth="1"/>
+    <col min="12" max="13" width="16.6640625" style="5" customWidth="1"/>
+    <col min="14" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="79"/>
-      <c r="B1" s="80"/>
-      <c r="C1" s="80"/>
-      <c r="D1" s="80"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="88" t="s">
+    <row r="1" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="74"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="83" t="s">
         <v>17</v>
       </c>
-      <c r="G1" s="89"/>
-      <c r="H1" s="89"/>
-      <c r="I1" s="89"/>
-      <c r="J1" s="89"/>
-      <c r="K1" s="90"/>
+      <c r="G1" s="84"/>
+      <c r="H1" s="84"/>
+      <c r="I1" s="84"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="85"/>
       <c r="L1" s="14" t="s">
         <v>6</v>
       </c>
@@ -1449,18 +1440,18 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="82"/>
-      <c r="B2" s="83"/>
-      <c r="C2" s="83"/>
-      <c r="D2" s="83"/>
-      <c r="E2" s="84"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="92"/>
-      <c r="H2" s="92"/>
-      <c r="I2" s="92"/>
-      <c r="J2" s="92"/>
-      <c r="K2" s="93"/>
+    <row r="2" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="77"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="87"/>
+      <c r="H2" s="87"/>
+      <c r="I2" s="87"/>
+      <c r="J2" s="87"/>
+      <c r="K2" s="88"/>
       <c r="L2" s="43" t="s">
         <v>7</v>
       </c>
@@ -1468,18 +1459,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="82"/>
-      <c r="B3" s="83"/>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="84"/>
-      <c r="F3" s="91"/>
-      <c r="G3" s="92"/>
-      <c r="H3" s="92"/>
-      <c r="I3" s="92"/>
-      <c r="J3" s="92"/>
-      <c r="K3" s="93"/>
+    <row r="3" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="77"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="79"/>
+      <c r="F3" s="86"/>
+      <c r="G3" s="87"/>
+      <c r="H3" s="87"/>
+      <c r="I3" s="87"/>
+      <c r="J3" s="87"/>
+      <c r="K3" s="88"/>
       <c r="L3" s="43" t="s">
         <v>10</v>
       </c>
@@ -1487,18 +1478,18 @@
         <v>44937</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="85"/>
-      <c r="B4" s="86"/>
-      <c r="C4" s="86"/>
-      <c r="D4" s="86"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="94"/>
-      <c r="G4" s="95"/>
-      <c r="H4" s="95"/>
-      <c r="I4" s="95"/>
-      <c r="J4" s="95"/>
-      <c r="K4" s="96"/>
+    <row r="4" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="80"/>
+      <c r="B4" s="81"/>
+      <c r="C4" s="81"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="82"/>
+      <c r="F4" s="89"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="91"/>
       <c r="L4" s="14" t="s">
         <v>8</v>
       </c>
@@ -1506,7 +1497,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A5" s="15"/>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
@@ -1521,45 +1512,45 @@
       <c r="L5" s="16"/>
       <c r="M5" s="16"/>
     </row>
-    <row r="6" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
         <v>19</v>
       </c>
       <c r="B6" s="20"/>
-      <c r="C6" s="104"/>
-      <c r="D6" s="104"/>
-      <c r="E6" s="104"/>
+      <c r="C6" s="94"/>
+      <c r="D6" s="94"/>
+      <c r="E6" s="94"/>
       <c r="F6" s="20"/>
       <c r="G6" s="20"/>
       <c r="H6" s="20"/>
       <c r="I6" s="20"/>
-      <c r="J6" s="98" t="s">
+      <c r="J6" s="92" t="s">
         <v>22</v>
       </c>
-      <c r="K6" s="98"/>
-      <c r="L6" s="59"/>
+      <c r="K6" s="92"/>
+      <c r="L6" s="53"/>
       <c r="M6" s="17"/>
     </row>
-    <row r="7" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="98" t="s">
+    <row r="7" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="92" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="98"/>
-      <c r="C7" s="104"/>
-      <c r="D7" s="104"/>
-      <c r="E7" s="104"/>
+      <c r="B7" s="92"/>
+      <c r="C7" s="94"/>
+      <c r="D7" s="94"/>
+      <c r="E7" s="94"/>
       <c r="F7" s="20"/>
       <c r="G7" s="20"/>
       <c r="H7" s="20"/>
       <c r="I7" s="20"/>
-      <c r="J7" s="98" t="s">
+      <c r="J7" s="92" t="s">
         <v>38</v>
       </c>
-      <c r="K7" s="98"/>
-      <c r="L7" s="60"/>
+      <c r="K7" s="92"/>
+      <c r="L7" s="54"/>
       <c r="M7" s="17"/>
     </row>
-    <row r="8" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="31"/>
       <c r="B8" s="31"/>
       <c r="C8" s="20"/>
@@ -1576,7 +1567,7 @@
       <c r="L8" s="17"/>
       <c r="M8" s="17"/>
     </row>
-    <row r="9" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="32" t="s">
         <v>21</v>
       </c>
@@ -1594,7 +1585,7 @@
       <c r="M9" s="35"/>
       <c r="N9" s="36"/>
     </row>
-    <row r="10" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="37" t="s">
         <v>12</v>
       </c>
@@ -1603,18 +1594,18 @@
         <v>0</v>
       </c>
       <c r="D10" s="37"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="61"/>
-      <c r="G10" s="61"/>
-      <c r="H10" s="61"/>
-      <c r="I10" s="61"/>
-      <c r="J10" s="61"/>
-      <c r="K10" s="61"/>
-      <c r="L10" s="36"/>
-      <c r="M10" s="36"/>
+      <c r="E10" s="95"/>
+      <c r="F10" s="55"/>
+      <c r="G10" s="55"/>
+      <c r="H10" s="55"/>
+      <c r="I10" s="55"/>
+      <c r="J10" s="55"/>
+      <c r="K10" s="55"/>
+      <c r="L10" s="95"/>
+      <c r="M10" s="95"/>
       <c r="N10" s="36"/>
     </row>
-    <row r="11" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="37" t="s">
         <v>11</v>
       </c>
@@ -1623,18 +1614,18 @@
         <v>0</v>
       </c>
       <c r="D11" s="37"/>
-      <c r="E11" s="36"/>
-      <c r="F11" s="61"/>
-      <c r="G11" s="61"/>
-      <c r="H11" s="61"/>
-      <c r="I11" s="61"/>
-      <c r="J11" s="61"/>
-      <c r="K11" s="61"/>
-      <c r="L11" s="36"/>
-      <c r="M11" s="36"/>
+      <c r="E11" s="95"/>
+      <c r="F11" s="55"/>
+      <c r="G11" s="55"/>
+      <c r="H11" s="55"/>
+      <c r="I11" s="55"/>
+      <c r="J11" s="55"/>
+      <c r="K11" s="55"/>
+      <c r="L11" s="95"/>
+      <c r="M11" s="95"/>
       <c r="N11" s="36"/>
     </row>
-    <row r="12" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="37" t="s">
         <v>4</v>
       </c>
@@ -1642,19 +1633,19 @@
       <c r="C12" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D12" s="100"/>
-      <c r="E12" s="100"/>
-      <c r="F12" s="100"/>
-      <c r="G12" s="61"/>
-      <c r="H12" s="61"/>
-      <c r="I12" s="61"/>
-      <c r="J12" s="61"/>
-      <c r="K12" s="61"/>
-      <c r="L12" s="36"/>
-      <c r="M12" s="36"/>
+      <c r="D12" s="93"/>
+      <c r="E12" s="93"/>
+      <c r="F12" s="93"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+      <c r="J12" s="55"/>
+      <c r="K12" s="55"/>
+      <c r="L12" s="95"/>
+      <c r="M12" s="95"/>
       <c r="N12" s="36"/>
     </row>
-    <row r="13" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="37" t="s">
         <v>14</v>
       </c>
@@ -1663,18 +1654,18 @@
         <v>0</v>
       </c>
       <c r="D13" s="37"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="61"/>
-      <c r="G13" s="61"/>
-      <c r="H13" s="61"/>
-      <c r="I13" s="61"/>
-      <c r="J13" s="61"/>
-      <c r="K13" s="61"/>
-      <c r="L13" s="36"/>
-      <c r="M13" s="36"/>
+      <c r="E13" s="95"/>
+      <c r="F13" s="55"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="55"/>
+      <c r="I13" s="55"/>
+      <c r="J13" s="55"/>
+      <c r="K13" s="55"/>
+      <c r="L13" s="95"/>
+      <c r="M13" s="95"/>
       <c r="N13" s="36"/>
     </row>
-    <row r="14" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="37" t="s">
         <v>5</v>
       </c>
@@ -1682,28 +1673,28 @@
       <c r="C14" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D14" s="68"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="61"/>
-      <c r="G14" s="61"/>
-      <c r="H14" s="61"/>
-      <c r="I14" s="61"/>
-      <c r="J14" s="62" t="s">
+      <c r="D14" s="96"/>
+      <c r="E14" s="95"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
+      <c r="J14" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="K14" s="40"/>
-      <c r="L14" s="61"/>
-      <c r="M14" s="61"/>
+      <c r="K14" s="97"/>
+      <c r="L14" s="55"/>
+      <c r="M14" s="55"/>
       <c r="N14" s="36"/>
     </row>
-    <row r="15" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="38" t="s">
         <v>13</v>
       </c>
       <c r="B15" s="38"/>
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
-      <c r="E15" s="35"/>
+      <c r="E15" s="98"/>
       <c r="F15" s="33"/>
       <c r="G15" s="33"/>
       <c r="H15" s="33"/>
@@ -1714,7 +1705,7 @@
       <c r="M15" s="33"/>
       <c r="N15" s="36"/>
     </row>
-    <row r="16" spans="1:14" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="37" t="s">
         <v>3</v>
       </c>
@@ -1723,40 +1714,40 @@
         <v>0</v>
       </c>
       <c r="D16" s="37"/>
-      <c r="E16" s="36"/>
-      <c r="F16" s="61"/>
-      <c r="G16" s="61"/>
-      <c r="H16" s="61"/>
-      <c r="I16" s="61"/>
-      <c r="J16" s="61"/>
-      <c r="K16" s="61"/>
-      <c r="L16" s="61"/>
-      <c r="M16" s="61"/>
+      <c r="E16" s="95"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="55"/>
+      <c r="H16" s="55"/>
+      <c r="I16" s="55"/>
+      <c r="J16" s="55"/>
+      <c r="K16" s="55"/>
+      <c r="L16" s="55"/>
+      <c r="M16" s="55"/>
       <c r="N16" s="36"/>
     </row>
-    <row r="17" spans="1:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="100" t="s">
+    <row r="17" spans="1:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="93" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="100"/>
+      <c r="B17" s="93"/>
       <c r="C17" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="D17" s="100"/>
-      <c r="E17" s="100"/>
-      <c r="F17" s="100"/>
-      <c r="G17" s="100"/>
-      <c r="H17" s="100"/>
-      <c r="I17" s="100"/>
-      <c r="J17" s="100"/>
-      <c r="K17" s="100"/>
-      <c r="L17" s="100"/>
-      <c r="M17" s="61"/>
-      <c r="N17" s="67" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D17" s="93"/>
+      <c r="E17" s="93"/>
+      <c r="F17" s="93"/>
+      <c r="G17" s="93"/>
+      <c r="H17" s="93"/>
+      <c r="I17" s="93"/>
+      <c r="J17" s="93"/>
+      <c r="K17" s="93"/>
+      <c r="L17" s="93"/>
+      <c r="M17" s="55"/>
+      <c r="N17" s="61" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="37" t="s">
         <v>1</v>
       </c>
@@ -1765,18 +1756,18 @@
         <v>0</v>
       </c>
       <c r="D18" s="37"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="63"/>
-      <c r="G18" s="61"/>
-      <c r="H18" s="61"/>
-      <c r="I18" s="61"/>
-      <c r="J18" s="61"/>
-      <c r="K18" s="61"/>
-      <c r="L18" s="61"/>
-      <c r="M18" s="61"/>
+      <c r="E18" s="95"/>
+      <c r="F18" s="57"/>
+      <c r="G18" s="55"/>
+      <c r="H18" s="55"/>
+      <c r="I18" s="55"/>
+      <c r="J18" s="55"/>
+      <c r="K18" s="55"/>
+      <c r="L18" s="55"/>
+      <c r="M18" s="55"/>
       <c r="N18" s="36"/>
     </row>
-    <row r="19" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="37" t="s">
         <v>2</v>
       </c>
@@ -1784,26 +1775,26 @@
       <c r="C19" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="D19" s="116"/>
-      <c r="E19" s="116"/>
-      <c r="F19" s="116"/>
-      <c r="G19" s="116"/>
-      <c r="H19" s="116"/>
-      <c r="I19" s="116"/>
-      <c r="J19" s="116"/>
-      <c r="K19" s="116"/>
-      <c r="L19" s="116"/>
-      <c r="M19" s="61"/>
+      <c r="D19" s="62"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="62"/>
+      <c r="G19" s="62"/>
+      <c r="H19" s="62"/>
+      <c r="I19" s="62"/>
+      <c r="J19" s="62"/>
+      <c r="K19" s="62"/>
+      <c r="L19" s="62"/>
+      <c r="M19" s="55"/>
       <c r="N19" s="36"/>
     </row>
-    <row r="20" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="48" t="s">
         <v>16</v>
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="19"/>
+      <c r="E20" s="99"/>
       <c r="F20" s="18"/>
       <c r="G20" s="21"/>
       <c r="H20" s="21"/>
@@ -1811,252 +1802,252 @@
       <c r="J20" s="21"/>
       <c r="K20" s="21"/>
       <c r="L20" s="21"/>
-      <c r="M20" s="19"/>
-    </row>
-    <row r="21" spans="1:14" ht="62.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M20" s="99"/>
+    </row>
+    <row r="21" spans="1:14" ht="62.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="22" t="s">
         <v>15</v>
       </c>
       <c r="B21" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="101" t="s">
+      <c r="C21" s="100" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="102"/>
-      <c r="E21" s="102"/>
-      <c r="F21" s="102"/>
-      <c r="G21" s="103"/>
-      <c r="H21" s="22" t="s">
+      <c r="D21" s="101"/>
+      <c r="E21" s="101"/>
+      <c r="F21" s="101"/>
+      <c r="G21" s="102"/>
+      <c r="H21" s="103" t="s">
         <v>34</v>
       </c>
-      <c r="I21" s="97" t="s">
+      <c r="I21" s="104" t="s">
         <v>31</v>
       </c>
-      <c r="J21" s="97"/>
-      <c r="K21" s="101" t="s">
+      <c r="J21" s="104"/>
+      <c r="K21" s="100" t="s">
         <v>32</v>
       </c>
-      <c r="L21" s="103"/>
-      <c r="M21" s="22" t="s">
+      <c r="L21" s="102"/>
+      <c r="M21" s="103" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="57">
+    <row r="22" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="51">
         <v>1</v>
       </c>
-      <c r="B22" s="66"/>
-      <c r="C22" s="76"/>
-      <c r="D22" s="77"/>
-      <c r="E22" s="77"/>
-      <c r="F22" s="77"/>
-      <c r="G22" s="78"/>
-      <c r="H22" s="58"/>
-      <c r="I22" s="99"/>
-      <c r="J22" s="99"/>
-      <c r="K22" s="70"/>
-      <c r="L22" s="71"/>
-      <c r="M22" s="56"/>
-    </row>
-    <row r="23" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="57"/>
-      <c r="B23" s="66"/>
-      <c r="C23" s="76"/>
-      <c r="D23" s="77"/>
-      <c r="E23" s="77"/>
-      <c r="F23" s="77"/>
-      <c r="G23" s="78"/>
-      <c r="H23" s="58"/>
-      <c r="I23" s="117"/>
-      <c r="J23" s="118"/>
-      <c r="K23" s="70"/>
-      <c r="L23" s="71"/>
-      <c r="M23" s="56"/>
-    </row>
-    <row r="24" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="57"/>
-      <c r="B24" s="66"/>
-      <c r="C24" s="76"/>
-      <c r="D24" s="77"/>
-      <c r="E24" s="77"/>
-      <c r="F24" s="77"/>
-      <c r="G24" s="78"/>
-      <c r="H24" s="58"/>
-      <c r="I24" s="117"/>
-      <c r="J24" s="118"/>
-      <c r="K24" s="70"/>
-      <c r="L24" s="71"/>
-      <c r="M24" s="56"/>
-    </row>
-    <row r="25" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="57"/>
-      <c r="B25" s="66"/>
-      <c r="C25" s="76"/>
-      <c r="D25" s="77"/>
-      <c r="E25" s="77"/>
-      <c r="F25" s="77"/>
-      <c r="G25" s="78"/>
-      <c r="H25" s="58"/>
-      <c r="I25" s="117"/>
-      <c r="J25" s="118"/>
-      <c r="K25" s="70"/>
-      <c r="L25" s="71"/>
-      <c r="M25" s="56"/>
-    </row>
-    <row r="26" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="57"/>
-      <c r="B26" s="66"/>
-      <c r="C26" s="76"/>
-      <c r="D26" s="77"/>
-      <c r="E26" s="77"/>
-      <c r="F26" s="77"/>
-      <c r="G26" s="78"/>
-      <c r="H26" s="58"/>
-      <c r="I26" s="117"/>
-      <c r="J26" s="118"/>
-      <c r="K26" s="70"/>
-      <c r="L26" s="71"/>
-      <c r="M26" s="56"/>
-    </row>
-    <row r="27" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="57"/>
-      <c r="B27" s="66"/>
-      <c r="C27" s="76"/>
-      <c r="D27" s="77"/>
-      <c r="E27" s="77"/>
-      <c r="F27" s="77"/>
-      <c r="G27" s="78"/>
-      <c r="H27" s="58"/>
-      <c r="I27" s="72"/>
-      <c r="J27" s="73"/>
-      <c r="K27" s="70"/>
-      <c r="L27" s="71"/>
-      <c r="M27" s="56"/>
-    </row>
-    <row r="28" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="57"/>
-      <c r="B28" s="66"/>
-      <c r="C28" s="69"/>
-      <c r="D28" s="69"/>
-      <c r="E28" s="69"/>
-      <c r="F28" s="69"/>
-      <c r="G28" s="69"/>
-      <c r="H28" s="58"/>
-      <c r="I28" s="72"/>
-      <c r="J28" s="73"/>
-      <c r="K28" s="74"/>
-      <c r="L28" s="75"/>
-      <c r="M28" s="56"/>
-    </row>
-    <row r="29" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="57"/>
-      <c r="B29" s="66"/>
-      <c r="C29" s="69"/>
-      <c r="D29" s="69"/>
-      <c r="E29" s="69"/>
-      <c r="F29" s="69"/>
-      <c r="G29" s="69"/>
-      <c r="H29" s="58"/>
-      <c r="I29" s="72"/>
-      <c r="J29" s="73"/>
-      <c r="K29" s="74"/>
-      <c r="L29" s="75"/>
-      <c r="M29" s="56"/>
-    </row>
-    <row r="30" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="57"/>
-      <c r="B30" s="66"/>
-      <c r="C30" s="69"/>
-      <c r="D30" s="69"/>
-      <c r="E30" s="69"/>
-      <c r="F30" s="69"/>
-      <c r="G30" s="69"/>
-      <c r="H30" s="58"/>
-      <c r="I30" s="72"/>
-      <c r="J30" s="73"/>
-      <c r="K30" s="74"/>
-      <c r="L30" s="75"/>
-      <c r="M30" s="56"/>
-    </row>
-    <row r="31" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="57"/>
-      <c r="B31" s="66"/>
-      <c r="C31" s="69"/>
-      <c r="D31" s="69"/>
-      <c r="E31" s="69"/>
-      <c r="F31" s="69"/>
-      <c r="G31" s="69"/>
-      <c r="H31" s="58"/>
-      <c r="I31" s="72"/>
-      <c r="J31" s="73"/>
-      <c r="K31" s="74"/>
-      <c r="L31" s="75"/>
-      <c r="M31" s="56"/>
-    </row>
-    <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="57"/>
-      <c r="B32" s="66"/>
-      <c r="C32" s="69"/>
-      <c r="D32" s="69"/>
-      <c r="E32" s="69"/>
-      <c r="F32" s="69"/>
-      <c r="G32" s="69"/>
-      <c r="H32" s="58"/>
-      <c r="I32" s="72"/>
-      <c r="J32" s="73"/>
-      <c r="K32" s="74"/>
-      <c r="L32" s="75"/>
-      <c r="M32" s="56"/>
-    </row>
-    <row r="33" spans="1:13" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="57"/>
-      <c r="B33" s="66"/>
-      <c r="C33" s="69"/>
-      <c r="D33" s="69"/>
-      <c r="E33" s="69"/>
-      <c r="F33" s="69"/>
-      <c r="G33" s="69"/>
-      <c r="H33" s="58"/>
-      <c r="I33" s="72"/>
-      <c r="J33" s="73"/>
-      <c r="K33" s="74"/>
-      <c r="L33" s="75"/>
-      <c r="M33" s="56"/>
-    </row>
-    <row r="34" spans="1:13" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="58"/>
-      <c r="B34" s="66"/>
-      <c r="C34" s="69"/>
-      <c r="D34" s="69"/>
-      <c r="E34" s="69"/>
-      <c r="F34" s="69"/>
-      <c r="G34" s="69"/>
-      <c r="H34" s="58"/>
-      <c r="I34" s="99"/>
-      <c r="J34" s="99"/>
-      <c r="K34" s="74"/>
-      <c r="L34" s="75"/>
-      <c r="M34" s="56"/>
-    </row>
-    <row r="35" spans="1:13" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="60"/>
+      <c r="C22" s="105"/>
+      <c r="D22" s="106"/>
+      <c r="E22" s="106"/>
+      <c r="F22" s="106"/>
+      <c r="G22" s="107"/>
+      <c r="H22" s="108"/>
+      <c r="I22" s="109"/>
+      <c r="J22" s="109"/>
+      <c r="K22" s="110"/>
+      <c r="L22" s="111"/>
+      <c r="M22" s="112"/>
+    </row>
+    <row r="23" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="51"/>
+      <c r="B23" s="60"/>
+      <c r="C23" s="105"/>
+      <c r="D23" s="106"/>
+      <c r="E23" s="106"/>
+      <c r="F23" s="106"/>
+      <c r="G23" s="107"/>
+      <c r="H23" s="108"/>
+      <c r="I23" s="113"/>
+      <c r="J23" s="114"/>
+      <c r="K23" s="110"/>
+      <c r="L23" s="111"/>
+      <c r="M23" s="112"/>
+    </row>
+    <row r="24" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="51"/>
+      <c r="B24" s="60"/>
+      <c r="C24" s="105"/>
+      <c r="D24" s="106"/>
+      <c r="E24" s="106"/>
+      <c r="F24" s="106"/>
+      <c r="G24" s="107"/>
+      <c r="H24" s="108"/>
+      <c r="I24" s="113"/>
+      <c r="J24" s="114"/>
+      <c r="K24" s="110"/>
+      <c r="L24" s="111"/>
+      <c r="M24" s="112"/>
+    </row>
+    <row r="25" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="51"/>
+      <c r="B25" s="60"/>
+      <c r="C25" s="105"/>
+      <c r="D25" s="106"/>
+      <c r="E25" s="106"/>
+      <c r="F25" s="106"/>
+      <c r="G25" s="107"/>
+      <c r="H25" s="108"/>
+      <c r="I25" s="113"/>
+      <c r="J25" s="114"/>
+      <c r="K25" s="110"/>
+      <c r="L25" s="111"/>
+      <c r="M25" s="112"/>
+    </row>
+    <row r="26" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="51"/>
+      <c r="B26" s="60"/>
+      <c r="C26" s="105"/>
+      <c r="D26" s="106"/>
+      <c r="E26" s="106"/>
+      <c r="F26" s="106"/>
+      <c r="G26" s="107"/>
+      <c r="H26" s="108"/>
+      <c r="I26" s="113"/>
+      <c r="J26" s="114"/>
+      <c r="K26" s="110"/>
+      <c r="L26" s="111"/>
+      <c r="M26" s="112"/>
+    </row>
+    <row r="27" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="51"/>
+      <c r="B27" s="60"/>
+      <c r="C27" s="105"/>
+      <c r="D27" s="106"/>
+      <c r="E27" s="106"/>
+      <c r="F27" s="106"/>
+      <c r="G27" s="107"/>
+      <c r="H27" s="108"/>
+      <c r="I27" s="115"/>
+      <c r="J27" s="116"/>
+      <c r="K27" s="110"/>
+      <c r="L27" s="111"/>
+      <c r="M27" s="112"/>
+    </row>
+    <row r="28" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="51"/>
+      <c r="B28" s="60"/>
+      <c r="C28" s="117"/>
+      <c r="D28" s="117"/>
+      <c r="E28" s="117"/>
+      <c r="F28" s="117"/>
+      <c r="G28" s="117"/>
+      <c r="H28" s="108"/>
+      <c r="I28" s="115"/>
+      <c r="J28" s="116"/>
+      <c r="K28" s="118"/>
+      <c r="L28" s="119"/>
+      <c r="M28" s="112"/>
+    </row>
+    <row r="29" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="51"/>
+      <c r="B29" s="60"/>
+      <c r="C29" s="117"/>
+      <c r="D29" s="117"/>
+      <c r="E29" s="117"/>
+      <c r="F29" s="117"/>
+      <c r="G29" s="117"/>
+      <c r="H29" s="108"/>
+      <c r="I29" s="115"/>
+      <c r="J29" s="116"/>
+      <c r="K29" s="118"/>
+      <c r="L29" s="119"/>
+      <c r="M29" s="112"/>
+    </row>
+    <row r="30" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="51"/>
+      <c r="B30" s="60"/>
+      <c r="C30" s="117"/>
+      <c r="D30" s="117"/>
+      <c r="E30" s="117"/>
+      <c r="F30" s="117"/>
+      <c r="G30" s="117"/>
+      <c r="H30" s="108"/>
+      <c r="I30" s="115"/>
+      <c r="J30" s="116"/>
+      <c r="K30" s="118"/>
+      <c r="L30" s="119"/>
+      <c r="M30" s="112"/>
+    </row>
+    <row r="31" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="51"/>
+      <c r="B31" s="60"/>
+      <c r="C31" s="117"/>
+      <c r="D31" s="117"/>
+      <c r="E31" s="117"/>
+      <c r="F31" s="117"/>
+      <c r="G31" s="117"/>
+      <c r="H31" s="108"/>
+      <c r="I31" s="115"/>
+      <c r="J31" s="116"/>
+      <c r="K31" s="118"/>
+      <c r="L31" s="119"/>
+      <c r="M31" s="112"/>
+    </row>
+    <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="51"/>
+      <c r="B32" s="60"/>
+      <c r="C32" s="117"/>
+      <c r="D32" s="117"/>
+      <c r="E32" s="117"/>
+      <c r="F32" s="117"/>
+      <c r="G32" s="117"/>
+      <c r="H32" s="108"/>
+      <c r="I32" s="115"/>
+      <c r="J32" s="116"/>
+      <c r="K32" s="118"/>
+      <c r="L32" s="119"/>
+      <c r="M32" s="112"/>
+    </row>
+    <row r="33" spans="1:13" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="51"/>
+      <c r="B33" s="60"/>
+      <c r="C33" s="117"/>
+      <c r="D33" s="117"/>
+      <c r="E33" s="117"/>
+      <c r="F33" s="117"/>
+      <c r="G33" s="117"/>
+      <c r="H33" s="108"/>
+      <c r="I33" s="115"/>
+      <c r="J33" s="116"/>
+      <c r="K33" s="118"/>
+      <c r="L33" s="119"/>
+      <c r="M33" s="112"/>
+    </row>
+    <row r="34" spans="1:13" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="52"/>
+      <c r="B34" s="60"/>
+      <c r="C34" s="117"/>
+      <c r="D34" s="117"/>
+      <c r="E34" s="117"/>
+      <c r="F34" s="117"/>
+      <c r="G34" s="117"/>
+      <c r="H34" s="108"/>
+      <c r="I34" s="109"/>
+      <c r="J34" s="109"/>
+      <c r="K34" s="118"/>
+      <c r="L34" s="119"/>
+      <c r="M34" s="112"/>
+    </row>
+    <row r="35" spans="1:13" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B35" s="27"/>
-      <c r="C35" s="51"/>
-      <c r="D35" s="52"/>
-      <c r="E35" s="53"/>
-      <c r="F35" s="53"/>
-      <c r="G35" s="53"/>
-      <c r="H35" s="54"/>
-      <c r="I35" s="53"/>
-      <c r="J35" s="53"/>
-      <c r="K35" s="55"/>
-      <c r="L35" s="55"/>
-      <c r="M35" s="55"/>
-    </row>
-    <row r="36" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C35" s="120"/>
+      <c r="D35" s="121"/>
+      <c r="E35" s="122"/>
+      <c r="F35" s="122"/>
+      <c r="G35" s="122"/>
+      <c r="H35" s="123"/>
+      <c r="I35" s="122"/>
+      <c r="J35" s="122"/>
+      <c r="K35" s="124"/>
+      <c r="L35" s="124"/>
+      <c r="M35" s="124"/>
+    </row>
+    <row r="36" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="27"/>
       <c r="C36" s="1"/>
@@ -2071,7 +2062,7 @@
       <c r="L36" s="26"/>
       <c r="M36" s="26"/>
     </row>
-    <row r="37" spans="1:13" ht="2.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="11"/>
       <c r="B37" s="12"/>
       <c r="C37" s="7"/>
@@ -2086,7 +2077,7 @@
       <c r="L37" s="10"/>
       <c r="M37" s="10"/>
     </row>
-    <row r="38" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="27" t="s">
         <v>24</v>
       </c>
@@ -2095,21 +2086,19 @@
       <c r="D38" s="23"/>
       <c r="E38" s="24"/>
       <c r="F38" s="24"/>
-      <c r="G38" s="108" t="s">
-        <v>43</v>
-      </c>
-      <c r="H38" s="106" t="s">
+      <c r="G38" s="66"/>
+      <c r="H38" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="I38" s="107"/>
+      <c r="I38" s="65"/>
       <c r="J38" s="24"/>
-      <c r="K38" s="111"/>
-      <c r="L38" s="109" t="s">
+      <c r="K38" s="69"/>
+      <c r="L38" s="67" t="s">
         <v>27</v>
       </c>
-      <c r="M38" s="110"/>
-    </row>
-    <row r="39" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M38" s="68"/>
+    </row>
+    <row r="39" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="42" t="s">
         <v>25</v>
       </c>
@@ -2118,15 +2107,15 @@
       <c r="D39" s="23"/>
       <c r="E39" s="24"/>
       <c r="F39" s="24"/>
-      <c r="G39" s="108"/>
-      <c r="H39" s="106"/>
-      <c r="I39" s="107"/>
+      <c r="G39" s="66"/>
+      <c r="H39" s="64"/>
+      <c r="I39" s="65"/>
       <c r="J39" s="24"/>
-      <c r="K39" s="111"/>
-      <c r="L39" s="109"/>
-      <c r="M39" s="110"/>
-    </row>
-    <row r="40" spans="1:13" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K39" s="69"/>
+      <c r="L39" s="67"/>
+      <c r="M39" s="68"/>
+    </row>
+    <row r="40" spans="1:13" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="27"/>
       <c r="B40" s="27"/>
       <c r="C40" s="23"/>
@@ -2141,7 +2130,7 @@
       <c r="L40" s="26"/>
       <c r="M40" s="26"/>
     </row>
-    <row r="41" spans="1:13" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="27" t="s">
         <v>28</v>
       </c>
@@ -2153,12 +2142,12 @@
       <c r="G41" s="24"/>
       <c r="H41" s="25"/>
       <c r="I41" s="24"/>
-      <c r="J41" s="113"/>
-      <c r="K41" s="113"/>
-      <c r="L41" s="113"/>
+      <c r="J41" s="71"/>
+      <c r="K41" s="71"/>
+      <c r="L41" s="71"/>
       <c r="M41" s="26"/>
     </row>
-    <row r="42" spans="1:13" ht="9.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:13" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="27"/>
       <c r="B42" s="27"/>
       <c r="C42" s="23"/>
@@ -2173,45 +2162,45 @@
       <c r="L42" s="24"/>
       <c r="M42" s="26"/>
     </row>
-    <row r="43" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="114" t="s">
+    <row r="43" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="72" t="s">
         <v>39</v>
       </c>
-      <c r="B43" s="114"/>
-      <c r="C43" s="64"/>
-      <c r="D43" s="64"/>
-      <c r="E43" s="64"/>
+      <c r="B43" s="72"/>
+      <c r="C43" s="58"/>
+      <c r="D43" s="58"/>
+      <c r="E43" s="58"/>
       <c r="F43" s="40"/>
       <c r="G43" s="40"/>
-      <c r="H43" s="112" t="s">
+      <c r="H43" s="70" t="s">
         <v>41</v>
       </c>
-      <c r="I43" s="112"/>
-      <c r="J43" s="64"/>
-      <c r="K43" s="65"/>
+      <c r="I43" s="70"/>
+      <c r="J43" s="58"/>
+      <c r="K43" s="59"/>
       <c r="L43" s="6"/>
       <c r="M43" s="6"/>
     </row>
-    <row r="44" spans="1:13" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="49" t="s">
         <v>40</v>
       </c>
       <c r="B44" s="50"/>
-      <c r="C44" s="64"/>
-      <c r="D44" s="64"/>
-      <c r="E44" s="64"/>
+      <c r="C44" s="58"/>
+      <c r="D44" s="58"/>
+      <c r="E44" s="58"/>
       <c r="F44" s="40"/>
       <c r="G44" s="41"/>
-      <c r="H44" s="115" t="s">
+      <c r="H44" s="73" t="s">
         <v>42</v>
       </c>
-      <c r="I44" s="115"/>
-      <c r="J44" s="64"/>
-      <c r="K44" s="65"/>
+      <c r="I44" s="73"/>
+      <c r="J44" s="58"/>
+      <c r="K44" s="59"/>
       <c r="L44" s="6"/>
       <c r="M44" s="19"/>
     </row>
-    <row r="45" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="30"/>
       <c r="B45" s="30"/>
       <c r="C45" s="28"/>
@@ -2226,40 +2215,57 @@
       <c r="L45" s="19"/>
       <c r="M45" s="19"/>
     </row>
-    <row r="46" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="105" t="s">
-        <v>45</v>
-      </c>
-      <c r="B46" s="105"/>
-      <c r="C46" s="105"/>
-      <c r="D46" s="105"/>
-      <c r="E46" s="105"/>
-      <c r="F46" s="105"/>
-      <c r="G46" s="105"/>
-      <c r="H46" s="105"/>
-      <c r="I46" s="105"/>
-      <c r="J46" s="105"/>
-      <c r="K46" s="105"/>
-      <c r="L46" s="105"/>
-      <c r="M46" s="105"/>
+    <row r="46" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="63" t="s">
+        <v>44</v>
+      </c>
+      <c r="B46" s="63"/>
+      <c r="C46" s="63"/>
+      <c r="D46" s="63"/>
+      <c r="E46" s="63"/>
+      <c r="F46" s="63"/>
+      <c r="G46" s="63"/>
+      <c r="H46" s="63"/>
+      <c r="I46" s="63"/>
+      <c r="J46" s="63"/>
+      <c r="K46" s="63"/>
+      <c r="L46" s="63"/>
+      <c r="M46" s="63"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="27hf8pv3PGDGh2VH3nZTV5/358x2zohOnXEVUzO021BcMX6vZDykC3sE17QSAJJRjBVNP/vmWEmY7MCqEnJYDA==" saltValue="bSAda6sN7sZiTJEl/IFlbw==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="62">
-    <mergeCell ref="D19:L19"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="C34:G34"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="C33:G33"/>
-    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="C29:G29"/>
+    <mergeCell ref="C30:G30"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="A1:E4"/>
+    <mergeCell ref="F1:K4"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D17:L17"/>
     <mergeCell ref="A46:M46"/>
     <mergeCell ref="I31:J31"/>
     <mergeCell ref="I32:J32"/>
@@ -2276,38 +2282,20 @@
     <mergeCell ref="H44:I44"/>
     <mergeCell ref="C31:G31"/>
     <mergeCell ref="K31:L31"/>
-    <mergeCell ref="A1:E4"/>
-    <mergeCell ref="F1:K4"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D17:L17"/>
-    <mergeCell ref="C29:G29"/>
-    <mergeCell ref="C30:G30"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="C33:G33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="D19:L19"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="I27:J27"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.59055118110236227" right="0.59055118110236227" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>

</xml_diff>

<commit_message>
fix(templates): actualizar plantillas de recepcion con contrasena oficial
</commit_message>
<xml_diff>
--- a/app/templates/Recepciones/F-LEM-P-01.04 V05 RECEPCIÓN DE MUESTRAS DE ROCA.xlsx
+++ b/app/templates/Recepciones/F-LEM-P-01.04 V05 RECEPCIÓN DE MUESTRAS DE ROCA.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F465790-13C5-47A2-A86E-4B7836BD021E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4E7E633-46A5-4F31-B441-1664CD89A215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -774,169 +774,204 @@
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -944,41 +979,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1420,19 +1420,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="74"/>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="83" t="s">
+      <c r="A1" s="85"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="94" t="s">
         <v>17</v>
       </c>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="J1" s="84"/>
-      <c r="K1" s="85"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
+      <c r="I1" s="95"/>
+      <c r="J1" s="95"/>
+      <c r="K1" s="96"/>
       <c r="L1" s="14" t="s">
         <v>6</v>
       </c>
@@ -1441,17 +1441,17 @@
       </c>
     </row>
     <row r="2" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="77"/>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="87"/>
-      <c r="H2" s="87"/>
-      <c r="I2" s="87"/>
-      <c r="J2" s="87"/>
-      <c r="K2" s="88"/>
+      <c r="A2" s="88"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="98"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="99"/>
       <c r="L2" s="43" t="s">
         <v>7</v>
       </c>
@@ -1460,17 +1460,17 @@
       </c>
     </row>
     <row r="3" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="77"/>
-      <c r="B3" s="78"/>
-      <c r="C3" s="78"/>
-      <c r="D3" s="78"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="86"/>
-      <c r="G3" s="87"/>
-      <c r="H3" s="87"/>
-      <c r="I3" s="87"/>
-      <c r="J3" s="87"/>
-      <c r="K3" s="88"/>
+      <c r="A3" s="88"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="89"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="97"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="99"/>
       <c r="L3" s="43" t="s">
         <v>10</v>
       </c>
@@ -1479,17 +1479,17 @@
       </c>
     </row>
     <row r="4" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="80"/>
-      <c r="B4" s="81"/>
-      <c r="C4" s="81"/>
-      <c r="D4" s="81"/>
-      <c r="E4" s="82"/>
-      <c r="F4" s="89"/>
-      <c r="G4" s="90"/>
-      <c r="H4" s="90"/>
-      <c r="I4" s="90"/>
-      <c r="J4" s="90"/>
-      <c r="K4" s="91"/>
+      <c r="A4" s="91"/>
+      <c r="B4" s="92"/>
+      <c r="C4" s="92"/>
+      <c r="D4" s="92"/>
+      <c r="E4" s="93"/>
+      <c r="F4" s="100"/>
+      <c r="G4" s="101"/>
+      <c r="H4" s="101"/>
+      <c r="I4" s="101"/>
+      <c r="J4" s="101"/>
+      <c r="K4" s="102"/>
       <c r="L4" s="14" t="s">
         <v>8</v>
       </c>
@@ -1517,36 +1517,36 @@
         <v>19</v>
       </c>
       <c r="B6" s="20"/>
-      <c r="C6" s="94"/>
-      <c r="D6" s="94"/>
-      <c r="E6" s="94"/>
+      <c r="C6" s="110"/>
+      <c r="D6" s="110"/>
+      <c r="E6" s="110"/>
       <c r="F6" s="20"/>
       <c r="G6" s="20"/>
       <c r="H6" s="20"/>
       <c r="I6" s="20"/>
-      <c r="J6" s="92" t="s">
+      <c r="J6" s="104" t="s">
         <v>22</v>
       </c>
-      <c r="K6" s="92"/>
+      <c r="K6" s="104"/>
       <c r="L6" s="53"/>
       <c r="M6" s="17"/>
     </row>
     <row r="7" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="92" t="s">
+      <c r="A7" s="104" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="92"/>
-      <c r="C7" s="94"/>
-      <c r="D7" s="94"/>
-      <c r="E7" s="94"/>
+      <c r="B7" s="104"/>
+      <c r="C7" s="110"/>
+      <c r="D7" s="110"/>
+      <c r="E7" s="110"/>
       <c r="F7" s="20"/>
       <c r="G7" s="20"/>
       <c r="H7" s="20"/>
       <c r="I7" s="20"/>
-      <c r="J7" s="92" t="s">
+      <c r="J7" s="104" t="s">
         <v>38</v>
       </c>
-      <c r="K7" s="92"/>
+      <c r="K7" s="104"/>
       <c r="L7" s="54"/>
       <c r="M7" s="17"/>
     </row>
@@ -1594,15 +1594,15 @@
         <v>0</v>
       </c>
       <c r="D10" s="37"/>
-      <c r="E10" s="95"/>
+      <c r="E10" s="62"/>
       <c r="F10" s="55"/>
       <c r="G10" s="55"/>
       <c r="H10" s="55"/>
       <c r="I10" s="55"/>
       <c r="J10" s="55"/>
       <c r="K10" s="55"/>
-      <c r="L10" s="95"/>
-      <c r="M10" s="95"/>
+      <c r="L10" s="62"/>
+      <c r="M10" s="62"/>
       <c r="N10" s="36"/>
     </row>
     <row r="11" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1614,15 +1614,15 @@
         <v>0</v>
       </c>
       <c r="D11" s="37"/>
-      <c r="E11" s="95"/>
+      <c r="E11" s="62"/>
       <c r="F11" s="55"/>
       <c r="G11" s="55"/>
       <c r="H11" s="55"/>
       <c r="I11" s="55"/>
       <c r="J11" s="55"/>
       <c r="K11" s="55"/>
-      <c r="L11" s="95"/>
-      <c r="M11" s="95"/>
+      <c r="L11" s="62"/>
+      <c r="M11" s="62"/>
       <c r="N11" s="36"/>
     </row>
     <row r="12" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1633,16 +1633,16 @@
       <c r="C12" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D12" s="93"/>
-      <c r="E12" s="93"/>
-      <c r="F12" s="93"/>
+      <c r="D12" s="106"/>
+      <c r="E12" s="106"/>
+      <c r="F12" s="106"/>
       <c r="G12" s="55"/>
       <c r="H12" s="55"/>
       <c r="I12" s="55"/>
       <c r="J12" s="55"/>
       <c r="K12" s="55"/>
-      <c r="L12" s="95"/>
-      <c r="M12" s="95"/>
+      <c r="L12" s="62"/>
+      <c r="M12" s="62"/>
       <c r="N12" s="36"/>
     </row>
     <row r="13" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1654,15 +1654,15 @@
         <v>0</v>
       </c>
       <c r="D13" s="37"/>
-      <c r="E13" s="95"/>
+      <c r="E13" s="62"/>
       <c r="F13" s="55"/>
       <c r="G13" s="55"/>
       <c r="H13" s="55"/>
       <c r="I13" s="55"/>
       <c r="J13" s="55"/>
       <c r="K13" s="55"/>
-      <c r="L13" s="95"/>
-      <c r="M13" s="95"/>
+      <c r="L13" s="62"/>
+      <c r="M13" s="62"/>
       <c r="N13" s="36"/>
     </row>
     <row r="14" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1673,8 +1673,8 @@
       <c r="C14" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="D14" s="96"/>
-      <c r="E14" s="95"/>
+      <c r="D14" s="63"/>
+      <c r="E14" s="62"/>
       <c r="F14" s="55"/>
       <c r="G14" s="55"/>
       <c r="H14" s="55"/>
@@ -1682,7 +1682,7 @@
       <c r="J14" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="K14" s="97"/>
+      <c r="K14" s="64"/>
       <c r="L14" s="55"/>
       <c r="M14" s="55"/>
       <c r="N14" s="36"/>
@@ -1694,7 +1694,7 @@
       <c r="B15" s="38"/>
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
-      <c r="E15" s="98"/>
+      <c r="E15" s="65"/>
       <c r="F15" s="33"/>
       <c r="G15" s="33"/>
       <c r="H15" s="33"/>
@@ -1714,7 +1714,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="37"/>
-      <c r="E16" s="95"/>
+      <c r="E16" s="62"/>
       <c r="F16" s="55"/>
       <c r="G16" s="55"/>
       <c r="H16" s="55"/>
@@ -1726,22 +1726,22 @@
       <c r="N16" s="36"/>
     </row>
     <row r="17" spans="1:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="93" t="s">
+      <c r="A17" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="93"/>
+      <c r="B17" s="106"/>
       <c r="C17" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="D17" s="93"/>
-      <c r="E17" s="93"/>
-      <c r="F17" s="93"/>
-      <c r="G17" s="93"/>
-      <c r="H17" s="93"/>
-      <c r="I17" s="93"/>
-      <c r="J17" s="93"/>
-      <c r="K17" s="93"/>
-      <c r="L17" s="93"/>
+      <c r="D17" s="106"/>
+      <c r="E17" s="106"/>
+      <c r="F17" s="106"/>
+      <c r="G17" s="106"/>
+      <c r="H17" s="106"/>
+      <c r="I17" s="106"/>
+      <c r="J17" s="106"/>
+      <c r="K17" s="106"/>
+      <c r="L17" s="106"/>
       <c r="M17" s="55"/>
       <c r="N17" s="61" t="s">
         <v>43</v>
@@ -1756,7 +1756,7 @@
         <v>0</v>
       </c>
       <c r="D18" s="37"/>
-      <c r="E18" s="95"/>
+      <c r="E18" s="62"/>
       <c r="F18" s="57"/>
       <c r="G18" s="55"/>
       <c r="H18" s="55"/>
@@ -1775,15 +1775,15 @@
       <c r="C19" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="D19" s="62"/>
-      <c r="E19" s="62"/>
-      <c r="F19" s="62"/>
-      <c r="G19" s="62"/>
-      <c r="H19" s="62"/>
-      <c r="I19" s="62"/>
-      <c r="J19" s="62"/>
-      <c r="K19" s="62"/>
-      <c r="L19" s="62"/>
+      <c r="D19" s="122"/>
+      <c r="E19" s="122"/>
+      <c r="F19" s="122"/>
+      <c r="G19" s="122"/>
+      <c r="H19" s="122"/>
+      <c r="I19" s="122"/>
+      <c r="J19" s="122"/>
+      <c r="K19" s="122"/>
+      <c r="L19" s="122"/>
       <c r="M19" s="55"/>
       <c r="N19" s="36"/>
     </row>
@@ -1794,7 +1794,7 @@
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="99"/>
+      <c r="E20" s="66"/>
       <c r="F20" s="18"/>
       <c r="G20" s="21"/>
       <c r="H20" s="21"/>
@@ -1802,7 +1802,7 @@
       <c r="J20" s="21"/>
       <c r="K20" s="21"/>
       <c r="L20" s="21"/>
-      <c r="M20" s="99"/>
+      <c r="M20" s="66"/>
     </row>
     <row r="21" spans="1:14" ht="62.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="22" t="s">
@@ -1811,25 +1811,25 @@
       <c r="B21" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="100" t="s">
+      <c r="C21" s="107" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="101"/>
-      <c r="E21" s="101"/>
-      <c r="F21" s="101"/>
-      <c r="G21" s="102"/>
-      <c r="H21" s="103" t="s">
+      <c r="D21" s="108"/>
+      <c r="E21" s="108"/>
+      <c r="F21" s="108"/>
+      <c r="G21" s="109"/>
+      <c r="H21" s="67" t="s">
         <v>34</v>
       </c>
-      <c r="I21" s="104" t="s">
+      <c r="I21" s="103" t="s">
         <v>31</v>
       </c>
-      <c r="J21" s="104"/>
-      <c r="K21" s="100" t="s">
+      <c r="J21" s="103"/>
+      <c r="K21" s="107" t="s">
         <v>32</v>
       </c>
-      <c r="L21" s="102"/>
-      <c r="M21" s="103" t="s">
+      <c r="L21" s="109"/>
+      <c r="M21" s="67" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1838,214 +1838,214 @@
         <v>1</v>
       </c>
       <c r="B22" s="60"/>
-      <c r="C22" s="105"/>
-      <c r="D22" s="106"/>
-      <c r="E22" s="106"/>
-      <c r="F22" s="106"/>
-      <c r="G22" s="107"/>
-      <c r="H22" s="108"/>
-      <c r="I22" s="109"/>
-      <c r="J22" s="109"/>
-      <c r="K22" s="110"/>
-      <c r="L22" s="111"/>
-      <c r="M22" s="112"/>
+      <c r="C22" s="82"/>
+      <c r="D22" s="83"/>
+      <c r="E22" s="83"/>
+      <c r="F22" s="83"/>
+      <c r="G22" s="84"/>
+      <c r="H22" s="68"/>
+      <c r="I22" s="105"/>
+      <c r="J22" s="105"/>
+      <c r="K22" s="76"/>
+      <c r="L22" s="77"/>
+      <c r="M22" s="69"/>
     </row>
     <row r="23" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="51"/>
       <c r="B23" s="60"/>
-      <c r="C23" s="105"/>
-      <c r="D23" s="106"/>
-      <c r="E23" s="106"/>
-      <c r="F23" s="106"/>
-      <c r="G23" s="107"/>
-      <c r="H23" s="108"/>
-      <c r="I23" s="113"/>
-      <c r="J23" s="114"/>
-      <c r="K23" s="110"/>
-      <c r="L23" s="111"/>
-      <c r="M23" s="112"/>
+      <c r="C23" s="82"/>
+      <c r="D23" s="83"/>
+      <c r="E23" s="83"/>
+      <c r="F23" s="83"/>
+      <c r="G23" s="84"/>
+      <c r="H23" s="68"/>
+      <c r="I23" s="123"/>
+      <c r="J23" s="124"/>
+      <c r="K23" s="76"/>
+      <c r="L23" s="77"/>
+      <c r="M23" s="69"/>
     </row>
     <row r="24" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="51"/>
       <c r="B24" s="60"/>
-      <c r="C24" s="105"/>
-      <c r="D24" s="106"/>
-      <c r="E24" s="106"/>
-      <c r="F24" s="106"/>
-      <c r="G24" s="107"/>
-      <c r="H24" s="108"/>
-      <c r="I24" s="113"/>
-      <c r="J24" s="114"/>
-      <c r="K24" s="110"/>
-      <c r="L24" s="111"/>
-      <c r="M24" s="112"/>
+      <c r="C24" s="82"/>
+      <c r="D24" s="83"/>
+      <c r="E24" s="83"/>
+      <c r="F24" s="83"/>
+      <c r="G24" s="84"/>
+      <c r="H24" s="68"/>
+      <c r="I24" s="123"/>
+      <c r="J24" s="124"/>
+      <c r="K24" s="76"/>
+      <c r="L24" s="77"/>
+      <c r="M24" s="69"/>
     </row>
     <row r="25" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="51"/>
       <c r="B25" s="60"/>
-      <c r="C25" s="105"/>
-      <c r="D25" s="106"/>
-      <c r="E25" s="106"/>
-      <c r="F25" s="106"/>
-      <c r="G25" s="107"/>
-      <c r="H25" s="108"/>
-      <c r="I25" s="113"/>
-      <c r="J25" s="114"/>
-      <c r="K25" s="110"/>
-      <c r="L25" s="111"/>
-      <c r="M25" s="112"/>
+      <c r="C25" s="82"/>
+      <c r="D25" s="83"/>
+      <c r="E25" s="83"/>
+      <c r="F25" s="83"/>
+      <c r="G25" s="84"/>
+      <c r="H25" s="68"/>
+      <c r="I25" s="123"/>
+      <c r="J25" s="124"/>
+      <c r="K25" s="76"/>
+      <c r="L25" s="77"/>
+      <c r="M25" s="69"/>
     </row>
     <row r="26" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="51"/>
       <c r="B26" s="60"/>
-      <c r="C26" s="105"/>
-      <c r="D26" s="106"/>
-      <c r="E26" s="106"/>
-      <c r="F26" s="106"/>
-      <c r="G26" s="107"/>
-      <c r="H26" s="108"/>
-      <c r="I26" s="113"/>
-      <c r="J26" s="114"/>
-      <c r="K26" s="110"/>
-      <c r="L26" s="111"/>
-      <c r="M26" s="112"/>
+      <c r="C26" s="82"/>
+      <c r="D26" s="83"/>
+      <c r="E26" s="83"/>
+      <c r="F26" s="83"/>
+      <c r="G26" s="84"/>
+      <c r="H26" s="68"/>
+      <c r="I26" s="123"/>
+      <c r="J26" s="124"/>
+      <c r="K26" s="76"/>
+      <c r="L26" s="77"/>
+      <c r="M26" s="69"/>
     </row>
     <row r="27" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="51"/>
       <c r="B27" s="60"/>
-      <c r="C27" s="105"/>
-      <c r="D27" s="106"/>
-      <c r="E27" s="106"/>
-      <c r="F27" s="106"/>
-      <c r="G27" s="107"/>
-      <c r="H27" s="108"/>
-      <c r="I27" s="115"/>
-      <c r="J27" s="116"/>
-      <c r="K27" s="110"/>
-      <c r="L27" s="111"/>
-      <c r="M27" s="112"/>
+      <c r="C27" s="82"/>
+      <c r="D27" s="83"/>
+      <c r="E27" s="83"/>
+      <c r="F27" s="83"/>
+      <c r="G27" s="84"/>
+      <c r="H27" s="68"/>
+      <c r="I27" s="78"/>
+      <c r="J27" s="79"/>
+      <c r="K27" s="76"/>
+      <c r="L27" s="77"/>
+      <c r="M27" s="69"/>
     </row>
     <row r="28" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="51"/>
       <c r="B28" s="60"/>
-      <c r="C28" s="117"/>
-      <c r="D28" s="117"/>
-      <c r="E28" s="117"/>
-      <c r="F28" s="117"/>
-      <c r="G28" s="117"/>
-      <c r="H28" s="108"/>
-      <c r="I28" s="115"/>
-      <c r="J28" s="116"/>
-      <c r="K28" s="118"/>
-      <c r="L28" s="119"/>
-      <c r="M28" s="112"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="75"/>
+      <c r="E28" s="75"/>
+      <c r="F28" s="75"/>
+      <c r="G28" s="75"/>
+      <c r="H28" s="68"/>
+      <c r="I28" s="78"/>
+      <c r="J28" s="79"/>
+      <c r="K28" s="80"/>
+      <c r="L28" s="81"/>
+      <c r="M28" s="69"/>
     </row>
     <row r="29" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="51"/>
       <c r="B29" s="60"/>
-      <c r="C29" s="117"/>
-      <c r="D29" s="117"/>
-      <c r="E29" s="117"/>
-      <c r="F29" s="117"/>
-      <c r="G29" s="117"/>
-      <c r="H29" s="108"/>
-      <c r="I29" s="115"/>
-      <c r="J29" s="116"/>
-      <c r="K29" s="118"/>
-      <c r="L29" s="119"/>
-      <c r="M29" s="112"/>
+      <c r="C29" s="75"/>
+      <c r="D29" s="75"/>
+      <c r="E29" s="75"/>
+      <c r="F29" s="75"/>
+      <c r="G29" s="75"/>
+      <c r="H29" s="68"/>
+      <c r="I29" s="78"/>
+      <c r="J29" s="79"/>
+      <c r="K29" s="80"/>
+      <c r="L29" s="81"/>
+      <c r="M29" s="69"/>
     </row>
     <row r="30" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="51"/>
       <c r="B30" s="60"/>
-      <c r="C30" s="117"/>
-      <c r="D30" s="117"/>
-      <c r="E30" s="117"/>
-      <c r="F30" s="117"/>
-      <c r="G30" s="117"/>
-      <c r="H30" s="108"/>
-      <c r="I30" s="115"/>
-      <c r="J30" s="116"/>
-      <c r="K30" s="118"/>
-      <c r="L30" s="119"/>
-      <c r="M30" s="112"/>
+      <c r="C30" s="75"/>
+      <c r="D30" s="75"/>
+      <c r="E30" s="75"/>
+      <c r="F30" s="75"/>
+      <c r="G30" s="75"/>
+      <c r="H30" s="68"/>
+      <c r="I30" s="78"/>
+      <c r="J30" s="79"/>
+      <c r="K30" s="80"/>
+      <c r="L30" s="81"/>
+      <c r="M30" s="69"/>
     </row>
     <row r="31" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="51"/>
       <c r="B31" s="60"/>
-      <c r="C31" s="117"/>
-      <c r="D31" s="117"/>
-      <c r="E31" s="117"/>
-      <c r="F31" s="117"/>
-      <c r="G31" s="117"/>
-      <c r="H31" s="108"/>
-      <c r="I31" s="115"/>
-      <c r="J31" s="116"/>
-      <c r="K31" s="118"/>
-      <c r="L31" s="119"/>
-      <c r="M31" s="112"/>
+      <c r="C31" s="75"/>
+      <c r="D31" s="75"/>
+      <c r="E31" s="75"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="68"/>
+      <c r="I31" s="78"/>
+      <c r="J31" s="79"/>
+      <c r="K31" s="80"/>
+      <c r="L31" s="81"/>
+      <c r="M31" s="69"/>
     </row>
     <row r="32" spans="1:14" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="51"/>
       <c r="B32" s="60"/>
-      <c r="C32" s="117"/>
-      <c r="D32" s="117"/>
-      <c r="E32" s="117"/>
-      <c r="F32" s="117"/>
-      <c r="G32" s="117"/>
-      <c r="H32" s="108"/>
-      <c r="I32" s="115"/>
-      <c r="J32" s="116"/>
-      <c r="K32" s="118"/>
-      <c r="L32" s="119"/>
-      <c r="M32" s="112"/>
+      <c r="C32" s="75"/>
+      <c r="D32" s="75"/>
+      <c r="E32" s="75"/>
+      <c r="F32" s="75"/>
+      <c r="G32" s="75"/>
+      <c r="H32" s="68"/>
+      <c r="I32" s="78"/>
+      <c r="J32" s="79"/>
+      <c r="K32" s="80"/>
+      <c r="L32" s="81"/>
+      <c r="M32" s="69"/>
     </row>
     <row r="33" spans="1:13" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="51"/>
       <c r="B33" s="60"/>
-      <c r="C33" s="117"/>
-      <c r="D33" s="117"/>
-      <c r="E33" s="117"/>
-      <c r="F33" s="117"/>
-      <c r="G33" s="117"/>
-      <c r="H33" s="108"/>
-      <c r="I33" s="115"/>
-      <c r="J33" s="116"/>
-      <c r="K33" s="118"/>
-      <c r="L33" s="119"/>
-      <c r="M33" s="112"/>
+      <c r="C33" s="75"/>
+      <c r="D33" s="75"/>
+      <c r="E33" s="75"/>
+      <c r="F33" s="75"/>
+      <c r="G33" s="75"/>
+      <c r="H33" s="68"/>
+      <c r="I33" s="78"/>
+      <c r="J33" s="79"/>
+      <c r="K33" s="80"/>
+      <c r="L33" s="81"/>
+      <c r="M33" s="69"/>
     </row>
     <row r="34" spans="1:13" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="52"/>
       <c r="B34" s="60"/>
-      <c r="C34" s="117"/>
-      <c r="D34" s="117"/>
-      <c r="E34" s="117"/>
-      <c r="F34" s="117"/>
-      <c r="G34" s="117"/>
-      <c r="H34" s="108"/>
-      <c r="I34" s="109"/>
-      <c r="J34" s="109"/>
-      <c r="K34" s="118"/>
-      <c r="L34" s="119"/>
-      <c r="M34" s="112"/>
+      <c r="C34" s="75"/>
+      <c r="D34" s="75"/>
+      <c r="E34" s="75"/>
+      <c r="F34" s="75"/>
+      <c r="G34" s="75"/>
+      <c r="H34" s="68"/>
+      <c r="I34" s="105"/>
+      <c r="J34" s="105"/>
+      <c r="K34" s="80"/>
+      <c r="L34" s="81"/>
+      <c r="M34" s="69"/>
     </row>
     <row r="35" spans="1:13" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B35" s="27"/>
-      <c r="C35" s="120"/>
-      <c r="D35" s="121"/>
-      <c r="E35" s="122"/>
-      <c r="F35" s="122"/>
-      <c r="G35" s="122"/>
-      <c r="H35" s="123"/>
-      <c r="I35" s="122"/>
-      <c r="J35" s="122"/>
-      <c r="K35" s="124"/>
-      <c r="L35" s="124"/>
-      <c r="M35" s="124"/>
+      <c r="C35" s="70"/>
+      <c r="D35" s="71"/>
+      <c r="E35" s="72"/>
+      <c r="F35" s="72"/>
+      <c r="G35" s="72"/>
+      <c r="H35" s="73"/>
+      <c r="I35" s="72"/>
+      <c r="J35" s="72"/>
+      <c r="K35" s="74"/>
+      <c r="L35" s="74"/>
+      <c r="M35" s="74"/>
     </row>
     <row r="36" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
@@ -2086,17 +2086,17 @@
       <c r="D38" s="23"/>
       <c r="E38" s="24"/>
       <c r="F38" s="24"/>
-      <c r="G38" s="66"/>
-      <c r="H38" s="64" t="s">
+      <c r="G38" s="114"/>
+      <c r="H38" s="112" t="s">
         <v>26</v>
       </c>
-      <c r="I38" s="65"/>
+      <c r="I38" s="113"/>
       <c r="J38" s="24"/>
-      <c r="K38" s="69"/>
-      <c r="L38" s="67" t="s">
+      <c r="K38" s="117"/>
+      <c r="L38" s="115" t="s">
         <v>27</v>
       </c>
-      <c r="M38" s="68"/>
+      <c r="M38" s="116"/>
     </row>
     <row r="39" spans="1:13" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="42" t="s">
@@ -2107,13 +2107,13 @@
       <c r="D39" s="23"/>
       <c r="E39" s="24"/>
       <c r="F39" s="24"/>
-      <c r="G39" s="66"/>
-      <c r="H39" s="64"/>
-      <c r="I39" s="65"/>
+      <c r="G39" s="114"/>
+      <c r="H39" s="112"/>
+      <c r="I39" s="113"/>
       <c r="J39" s="24"/>
-      <c r="K39" s="69"/>
-      <c r="L39" s="67"/>
-      <c r="M39" s="68"/>
+      <c r="K39" s="117"/>
+      <c r="L39" s="115"/>
+      <c r="M39" s="116"/>
     </row>
     <row r="40" spans="1:13" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="27"/>
@@ -2142,9 +2142,9 @@
       <c r="G41" s="24"/>
       <c r="H41" s="25"/>
       <c r="I41" s="24"/>
-      <c r="J41" s="71"/>
-      <c r="K41" s="71"/>
-      <c r="L41" s="71"/>
+      <c r="J41" s="119"/>
+      <c r="K41" s="119"/>
+      <c r="L41" s="119"/>
       <c r="M41" s="26"/>
     </row>
     <row r="42" spans="1:13" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2163,19 +2163,19 @@
       <c r="M42" s="26"/>
     </row>
     <row r="43" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="72" t="s">
+      <c r="A43" s="120" t="s">
         <v>39</v>
       </c>
-      <c r="B43" s="72"/>
+      <c r="B43" s="120"/>
       <c r="C43" s="58"/>
       <c r="D43" s="58"/>
       <c r="E43" s="58"/>
       <c r="F43" s="40"/>
       <c r="G43" s="40"/>
-      <c r="H43" s="70" t="s">
+      <c r="H43" s="118" t="s">
         <v>41</v>
       </c>
-      <c r="I43" s="70"/>
+      <c r="I43" s="118"/>
       <c r="J43" s="58"/>
       <c r="K43" s="59"/>
       <c r="L43" s="6"/>
@@ -2191,10 +2191,10 @@
       <c r="E44" s="58"/>
       <c r="F44" s="40"/>
       <c r="G44" s="41"/>
-      <c r="H44" s="73" t="s">
+      <c r="H44" s="121" t="s">
         <v>42</v>
       </c>
-      <c r="I44" s="73"/>
+      <c r="I44" s="121"/>
       <c r="J44" s="58"/>
       <c r="K44" s="59"/>
       <c r="L44" s="6"/>
@@ -2216,24 +2216,71 @@
       <c r="M45" s="19"/>
     </row>
     <row r="46" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="63" t="s">
+      <c r="A46" s="111" t="s">
         <v>44</v>
       </c>
-      <c r="B46" s="63"/>
-      <c r="C46" s="63"/>
-      <c r="D46" s="63"/>
-      <c r="E46" s="63"/>
-      <c r="F46" s="63"/>
-      <c r="G46" s="63"/>
-      <c r="H46" s="63"/>
-      <c r="I46" s="63"/>
-      <c r="J46" s="63"/>
-      <c r="K46" s="63"/>
-      <c r="L46" s="63"/>
-      <c r="M46" s="63"/>
+      <c r="B46" s="111"/>
+      <c r="C46" s="111"/>
+      <c r="D46" s="111"/>
+      <c r="E46" s="111"/>
+      <c r="F46" s="111"/>
+      <c r="G46" s="111"/>
+      <c r="H46" s="111"/>
+      <c r="I46" s="111"/>
+      <c r="J46" s="111"/>
+      <c r="K46" s="111"/>
+      <c r="L46" s="111"/>
+      <c r="M46" s="111"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="UfKSSNTvHvvB8e+cTv8tl4TNhNvvBV8qAuBFwYGuLvQRSh1lMWBfH7Ri3gBs1EyV4Myw5pKeallxfuFgPddEdQ==" saltValue="3X7+01y1cqH63WW/s1YgBA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="62">
+    <mergeCell ref="D19:L19"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="C33:G33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="A46:M46"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="H38:I39"/>
+    <mergeCell ref="G38:G39"/>
+    <mergeCell ref="L38:M39"/>
+    <mergeCell ref="K38:K39"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="J41:L41"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="H44:I44"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="A1:E4"/>
+    <mergeCell ref="F1:K4"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D17:L17"/>
     <mergeCell ref="C29:G29"/>
     <mergeCell ref="C30:G30"/>
     <mergeCell ref="K23:L23"/>
@@ -2250,52 +2297,6 @@
     <mergeCell ref="C23:G23"/>
     <mergeCell ref="C24:G24"/>
     <mergeCell ref="C25:G25"/>
-    <mergeCell ref="A1:E4"/>
-    <mergeCell ref="F1:K4"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D17:L17"/>
-    <mergeCell ref="A46:M46"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="H38:I39"/>
-    <mergeCell ref="G38:G39"/>
-    <mergeCell ref="L38:M39"/>
-    <mergeCell ref="K38:K39"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="J41:L41"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="H44:I44"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="C34:G34"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="C33:G33"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="D19:L19"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="I27:J27"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.59055118110236227" right="0.59055118110236227" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>

</xml_diff>